<commit_message>
Change preferred start times from 9/10/11 to 8/9/10 in sample data
Updated preferences.xlsx so the three start time groups are 08:00,
09:00, and 10:00 instead of the previous 09:00, 10:00, and 11:00.

https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/preferences.xlsx
+++ b/src/main/resources/sample-data/preferences.xlsx
@@ -499,7 +499,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -531,7 +531,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -2803,7 +2803,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add 20 agents to preferences.xlsx to align with 120-agent mock data
Extended the sample preferences spreadsheet from 100 to 120 agents,
matching the new names added to MockBambooHRClient (Alice through Tobias).
Start times distributed across 08:00, 09:00, and 10:00 to balance shifts.

https://claude.ai/code/session_01FRL5mvLBGhucHuBvGc1oVJ
</commit_message>
<xml_diff>
--- a/src/main/resources/sample-data/preferences.xlsx
+++ b/src/main/resources/sample-data/preferences.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -3676,6 +3676,646 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Alice Smith</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>alice.smith101@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Brian Johnson</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>brian.johnson102@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Catherine Williams</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>catherine.williams103@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Derek Brown</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>derek.brown104@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Elena Jones</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>elena.jones105@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Felix Garcia</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>felix.garcia106@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Georgia Miller</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>georgia.miller107@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Hugo Davis</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>hugo.davis108@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Iris Rodriguez</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>iris.rodriguez109@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Julian Martinez</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>julian.martinez110@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Katherine Hernandez</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>katherine.hernandez111@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Lorenzo Lopez</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>lorenzo.lopez112@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Madeline Gonzalez</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>madeline.gonzalez113@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Nico Wilson</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>nico.wilson114@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Ophelia Anderson</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>ophelia.anderson115@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Patrick Thomas</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>patrick.thomas116@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Quinn Taylor</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>quinn.taylor117@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Regina Moore</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>regina.moore118@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Sienna Jackson</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>sienna.jackson119@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Tobias Martin</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>tobias.martin120@vinted.example.com</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>MONDAY</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>